<commit_message>
2026-07-27: SLA% scope fixes, history chart timezone fix, KPI delta display, modal on-demand fetch, project memory docs
</commit_message>
<xml_diff>
--- a/docs/SLA_Dashboard_Tooltips.xlsx
+++ b/docs/SLA_Dashboard_Tooltips.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mortgageezy-my.sharepoint.com/personal/ntruong_mezy_com_au/Documents/Project_VibeCoding/SLA Dashboard/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_F3B0D10FEB2742546C1204628016A7F5C0207633" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8FA1FFC6-6DD6-4E59-8DB0-A173B9F5901F}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="11_B2309426A12742546C92895A7C17B4F5C0207261" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDBE9742-C192-4D07-82A0-D23EBAE6CCC3}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="102">
   <si>
     <t>Section</t>
   </si>
@@ -56,12 +56,12 @@
 Date basis: Date Created.</t>
   </si>
   <si>
-    <t>Count of ACTIVE tasks across all teams now._x000D_
-_x000D_
-Includes: In Progress, On Hold, On Queue, Not Queued._x000D_
-_x000D_
-Excluded: Completed and Cancelled._x000D_
-_x000D_
+    <t>Count of ACTIVE tasks across all teams now._x000D__x000D_
+_x000D__x000D_
+Includes: In Progress, On Hold, On Queue, Not Queued._x000D__x000D_
+_x000D__x000D_
+Excluded: Completed and Cancelled._x000D__x000D_
+_x000D__x000D_
 Date basis: Date Created.</t>
   </si>
   <si>
@@ -73,21 +73,21 @@
   <si>
     <t>SLA compliance rate % - For COMPLETED tasks only 
 Formula: 
-[Total On-time# + Total Overdue #] ÷ total completed # × 100
+[Total On-time# + Total Overdue #] / total completed # * 100
 Includes: Completed.
 Excluded: Active and Cancelled.
 Date basis: Date Created.</t>
   </si>
   <si>
-    <t>SLA compliance rate % - For COMPLETED tasks only _x000D_
-_x000D_
-Formula: _x000D_
-[Total On-time# + Total Overdue #] ÷ total completed # × 100_x000D_
-_x000D_
-Includes: Completed._x000D_
-_x000D_
-Excluded: Active and Cancelled._x000D_
-_x000D_
+    <t>SLA compliance rate % - For COMPLETED tasks only _x000D__x000D_
+_x000D__x000D_
+Formula: _x000D__x000D_
+[Total On-time# + Total Overdue #] ÷ total completed # × 100_x000D__x000D_
+_x000D__x000D_
+Includes: Completed._x000D__x000D_
+_x000D__x000D_
+Excluded: Active and Cancelled._x000D__x000D_
+_x000D__x000D_
 Date basis: Date Created.</t>
   </si>
   <si>
@@ -97,44 +97,37 @@
     <t>Dashboard → KPI tile: Avg Turnaround</t>
   </si>
   <si>
-    <t>Average TAT of ACTIVE tasks (current of all performance team cards) 
-Rules:
-- avg TAT = avg TotalHoursOnTask when not null
-Includes: Completed
-Excluded: Tasks where TotalHoursOnTask is null are excuded from the average
-Date basis: Date Created.</t>
-  </si>
-  <si>
-    <t>kpi.totalOverdue</t>
-  </si>
-  <si>
-    <t>Dashboard → KPI tile: Overdue</t>
-  </si>
-  <si>
-    <t>Count of active tasks that have exceeded their SLA target.
-Rules:
-- Overdue when TotalHoursOnTask &gt; SLAInHours
-- Overdue when  Current time &gt; SLAAdjustedDate 
-- Overdue when TotalHoursOnTask&gt; SLA target hours in Setting tab
-Includes: Active
-Excluded: Cancelled; Completed tasks; Tasks where TotalHoursOnTask is null or = 0
-Date basis: Date Created.
-Target is configurable per team In Settings.</t>
-  </si>
-  <si>
-    <t>Count of active tasks that have exceeded their SLA target._x000D_
+    <t>Average TAT of ACTIVE tasks _x000D_
 _x000D_
 Rules:_x000D_
-- Overdue when TotalHoursOnTask &gt; SLAInHours_x000D_
-- Overdue when  Current time &gt; SLAAdjustedDate _x000D_
-- Overdue when TotalHoursOnTask&gt; SLA target hours in Setting tab_x000D_
+- avg TAT = avg TotalHoursOnTask _x000D_
 _x000D_
 Includes: Active_x000D_
 _x000D_
-Excluded: Cancelled; Completed tasks; Tasks where TotalHoursOnTask is null or = 0_x000D_
+Excluded: Tasks where TotalHoursOnTask is null are excluded from the average_x000D_
 _x000D_
-Date basis: Date Created._x000D_
-_x000D_
+Date basis: Date Created.</t>
+  </si>
+  <si>
+    <t>kpi.totalOverdue</t>
+  </si>
+  <si>
+    <t>Dashboard → KPI tile: Overdue</t>
+  </si>
+  <si>
+    <t>Count of active tasks that have exceeded their SLA target._x000D__x000D_
+_x000D__x000D_
+Rules:_x000D__x000D_
+- Overdue when TotalHoursOnTask &gt; SLAInHours_x000D__x000D_
+- Overdue when  Current time &gt; SLAAdjustedDate _x000D__x000D_
+- Overdue when TotalHoursOnTask&gt; SLA target hours in Setting tab_x000D__x000D_
+_x000D__x000D_
+Includes: Active_x000D__x000D_
+_x000D__x000D_
+Excluded: Cancelled; Completed tasks; Tasks where TotalHoursOnTask is null or = 0_x000D__x000D_
+_x000D__x000D_
+Date basis: Date Created._x000D__x000D_
+_x000D__x000D_
 Target is configurable per team In Settings.</t>
   </si>
   <si>
@@ -153,12 +146,12 @@
 Date basis: Date Created.</t>
   </si>
   <si>
-    <t>Number of ACTIVE tasks currently in this team's queue._x000D_
-_x000D_
-Includes: In Progress, On Hold, On Queue, Not Queued._x000D_
-_x000D_
-Excluded: Completed and Cancelled._x000D_
-_x000D_
+    <t>Number of ACTIVE tasks currently in this team's queue._x000D__x000D_
+_x000D__x000D_
+Includes: In Progress, On Hold, On Queue, Not Queued._x000D__x000D_
+_x000D__x000D_
+Excluded: Completed and Cancelled._x000D__x000D_
+_x000D__x000D_
 Date basis: Date Created.</t>
   </si>
   <si>
@@ -170,37 +163,49 @@
   <si>
     <t>SLA compliance rate % - For COMPLETED tasks only 
 Formula: 
-[Total On-time# + Total Overdue #] ÷ total completed # × 100
+[Total On-time# + Total Overdue #] / total completed # * 100
 Rules:
-- Green ≥ 90% (On Target) 
-- Amber 75–89% (At Risk) 
+- Green &gt;= 90% (On Target)
+- Amber 75-89% (At Risk)
 - Red &lt; 75% (Breach)
 Includes: Completed.
 Excluded: Active and Cancelled.
 Date basis: Date Created.</t>
   </si>
   <si>
-    <t>SLA compliance rate % - For COMPLETED tasks only _x000D_
-_x000D_
-Formula: _x000D_
-[Total On-time# + Total Overdue #] ÷ total completed # × 100_x000D_
+    <t>SLA compliance rate % - For COMPLETED tasks only _x000D__x000D_
+_x000D__x000D_
+Formula: _x000D__x000D_
+[Total On-time# + Total Overdue #] ÷ total completed # × 100_x000D__x000D_
+_x000D__x000D_
+Rules:_x000D__x000D_
+- Green ≥ 90% (On Target) _x000D__x000D_
+- Amber 75–89% (At Risk) _x000D__x000D_
+- Red &lt; 75% (Breach)_x000D__x000D_
+_x000D__x000D_
+Includes: Completed._x000D__x000D_
+_x000D__x000D_
+Excluded: Active and Cancelled._x000D__x000D_
+_x000D__x000D_
+Date basis: Date Created.</t>
+  </si>
+  <si>
+    <t>team.avgTat</t>
+  </si>
+  <si>
+    <t>Dashboard → Team card: Avg TAT chip</t>
+  </si>
+  <si>
+    <t>Average TAT of ACTIVE tasks_x000D_
 _x000D_
 Rules:_x000D_
-- Green ≥ 90% (On Target) _x000D_
-- Amber 75–89% (At Risk) _x000D_
-- Red &lt; 75% (Breach)_x000D_
+- avg TAT = avg TotalHoursOnTask _x000D_
 _x000D_
-Includes: Completed._x000D_
+Includes: Active_x000D_
 _x000D_
-Excluded: Active and Cancelled._x000D_
+Excluded: Tasks where TotalHoursOnTask is null are excluded from the average_x000D_
 _x000D_
 Date basis: Date Created.</t>
-  </si>
-  <si>
-    <t>team.avgTat</t>
-  </si>
-  <si>
-    <t>Dashboard → Team card: Avg TAT chip</t>
   </si>
   <si>
     <t>team.overdue</t>
@@ -229,18 +234,18 @@
 - Hover over the chart to compare values on a specific day.</t>
   </si>
   <si>
-    <t>Rules:_x000D_
-- Business days only (weekends excluded)._x000D_
-- Each point = % of completed tasks SLA-compliant that day._x000D_
-_x000D_
-Includes: Completed tasks._x000D_
-_x000D_
-Excluded: Active and Cancelled tasks._x000D_
-_x000D_
-Date basis: Date Created._x000D_
-_x000D_
-Interactions:_x000D_
-- Click a team name in the legend to show or hide its line._x000D_
+    <t>Rules:_x000D__x000D_
+- Business days only (weekends excluded)._x000D__x000D_
+- Each point = % of completed tasks SLA-compliant that day._x000D__x000D_
+_x000D__x000D_
+Includes: Completed tasks._x000D__x000D_
+_x000D__x000D_
+Excluded: Active and Cancelled tasks._x000D__x000D_
+_x000D__x000D_
+Date basis: Date Created._x000D__x000D_
+_x000D__x000D_
+Interactions:_x000D__x000D_
+- Click a team name in the legend to show or hide its line._x000D__x000D_
 - Hover over the chart to compare values on a specific day.</t>
   </si>
   <si>
@@ -259,13 +264,13 @@
     <t>Teams tab → Status column header</t>
   </si>
   <si>
-    <t>● On Target — SLA ≥ 90%
-● At Risk — SLA 75–89%
-● Breach — SLA &lt; 75%</t>
-  </si>
-  <si>
-    <t>● On Target — SLA ≥ 90%_x000D_
-● At Risk — SLA 75–89%_x000D_
+    <t>On Target - SLA &gt;= 90%
+At Risk   - SLA 75-89%
+Breach    - SLA &lt; 75%</t>
+  </si>
+  <si>
+    <t>● On Target — SLA ≥ 90%_x000D__x000D_
+● At Risk — SLA 75–89%_x000D__x000D_
 ● Breach — SLA &lt; 75%</t>
   </si>
   <si>
@@ -290,12 +295,12 @@
 Date basis: Date Created.</t>
   </si>
   <si>
-    <t>Total ACTIVE tasks currently in this team's queue._x000D_
-_x000D_
-Includes: In Progress, On Hold, On Queue, Not Queued._x000D_
-_x000D_
-Excluded: Completed and Cancelled._x000D_
-_x000D_
+    <t>Total ACTIVE tasks currently in this team's queue._x000D__x000D_
+_x000D__x000D_
+Includes: In Progress, On Hold, On Queue, Not Queued._x000D__x000D_
+_x000D__x000D_
+Excluded: Completed and Cancelled._x000D__x000D_
+_x000D__x000D_
 Date basis: Date Created.</t>
   </si>
   <si>
@@ -305,52 +310,59 @@
     <t>Task Modal → Avg TAT chip (active tasks mode)</t>
   </si>
   <si>
-    <t>modal.avgTatCompleted</t>
-  </si>
-  <si>
-    <t>Task Modal → Avg TAT chip (completed tasks mode — SLA % badge click)</t>
-  </si>
-  <si>
-    <t>Average TAT across completed tasks 
-Rules:
-- avg TAT = avg TotalHoursOnTask when not null
-- DATEDIFF(DateCreated, DateCompleted) in hours when TotalHoursOnTask is null and SLAAdjustedDate is set
-Includes: Completed
-Excluded: Tasks where TotalHoursOnTask is null and SLAAdjustedDate is null
-Date basis: Date Created.</t>
-  </si>
-  <si>
-    <t>modal.overdue</t>
-  </si>
-  <si>
-    <t>Task Modal → Overdue chip (active tasks mode)</t>
-  </si>
-  <si>
-    <t>modal.overdueCompleted</t>
-  </si>
-  <si>
-    <t>Task Modal → Overdue (Only Completed Tasks) chip (completed tasks mode)</t>
-  </si>
-  <si>
-    <t>Count of completed tasks that exceeded their SLA target.
-Rules:
-- Overdue when TotalHoursOnTask &gt; SLAInHours
-- Overdue when DateCompleted &gt; SLAAdjustedDate
-Includes: Completed
-Excluded: Cancelled; Active tasks; Tasks where TotalHoursOnTask is null or = 0
-Date basis: Date Created</t>
-  </si>
-  <si>
-    <t>Count of completed tasks that exceeded their SLA target._x000D_
+    <t>Average TAT of ACTIVE tasks _x000D_
 _x000D_
 Rules:_x000D_
-- Overdue when TotalHoursOnTask &gt; SLAInHours_x000D_
-- Overdue when DateCompleted &gt; SLAAdjustedDate_x000D_
+- avg TAT = avg TotalHoursOnTask_x000D_
 _x000D_
 Includes: Completed_x000D_
 _x000D_
-Excluded: Cancelled; Active tasks; Tasks where TotalHoursOnTask is null or = 0_x000D_
+Excluded: Tasks where TotalHoursOnTask is null are excluded from the average_x000D_
 _x000D_
+Date basis: Date Created.</t>
+  </si>
+  <si>
+    <t>modal.avgTatCompleted</t>
+  </si>
+  <si>
+    <t>Task Modal → Avg TAT chip (completed tasks mode — SLA % badge click)</t>
+  </si>
+  <si>
+    <t>Average TAT across completed tasks _x000D_
+_x000D_
+Rules:_x000D_
+- avg TAT = avg TotalHoursOnTask when not null_x000D_
+- DateDiff (DateCreated, DateCompleted) in hours when TotalHoursOnTask is null and SLAAdjustedDate is set_x000D_
+_x000D_
+Includes: Completed_x000D_
+_x000D_
+Excluded: Tasks where TotalHoursOnTask is null and SLAAdjustedDate is null_x000D_
+_x000D_
+Date basis: Date Created.</t>
+  </si>
+  <si>
+    <t>modal.overdue</t>
+  </si>
+  <si>
+    <t>Task Modal → Overdue chip (active tasks mode)</t>
+  </si>
+  <si>
+    <t>modal.overdueCompleted</t>
+  </si>
+  <si>
+    <t>Task Modal → Overdue (Only Completed Tasks) chip (completed tasks mode)</t>
+  </si>
+  <si>
+    <t>Count of completed tasks that exceeded their SLA target._x000D__x000D_
+_x000D__x000D_
+Rules:_x000D__x000D_
+- Overdue when TotalHoursOnTask &gt; SLAInHours_x000D__x000D_
+- Overdue when DateCompleted &gt; SLAAdjustedDate_x000D__x000D_
+_x000D__x000D_
+Includes: Completed_x000D__x000D_
+_x000D__x000D_
+Excluded: Cancelled; Active tasks; Tasks where TotalHoursOnTask is null or = 0_x000D__x000D_
+_x000D__x000D_
 Date basis: Date Created</t>
   </si>
   <si>
@@ -363,18 +375,17 @@
     <t>Dashboard → Active Alerts panel title / Alerts tab title</t>
   </si>
   <si>
-    <t xml:space="preserve">1. For every team, the system counts how many of today's active tasks (In Progress, On Hold, On Queue, Not Queued) are compliant — meaning their elapsed time hasn't exceeded the task's own SLAInHours limit.
+    <t>1. For every team, the system counts how many of today's active tasks (In Progress, On Hold, On Queue, Not Queued) are compliant - meaning their elapsed time has not exceeded the task's own SLAInHours limit.
 2. It divides that by the total active task count to get a live SLA% for each team.
-3. Alerts clear automatically the next time the cache refreshes (every 5 min) if the team's SLA% has recovered above the threshold. No manual dismissal needed — though users can manually dismiss from the UI to hide it for their session.
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. For every team, the system counts how many of today's active tasks (In Progress, On Hold, On Queue, Not Queued) are compliant — meaning their elapsed time hasn't exceeded the task's own SLAInHours limit._x000D_
-_x000D_
-2. It divides that by the total active task count to get a live SLA% for each team._x000D_
-_x000D_
-3. Alerts clear automatically the next time the cache refreshes (every 5 min) if the team's SLA% has recovered above the threshold. No manual dismissal needed — though users can manually dismiss from the UI to hide it for their session._x000D_
-_x000D_
+3. Alerts clear automatically the next time the cache refreshes (every 5 min) if the team's SLA% has recovered above the threshold. No manual dismissal needed - though users can manually dismiss from the UI to hide it for their session.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. For every team, the system counts how many of today's active tasks (In Progress, On Hold, On Queue, Not Queued) are compliant — meaning their elapsed time hasn't exceeded the task's own SLAInHours limit._x000D__x000D_
+_x000D__x000D_
+2. It divides that by the total active task count to get a live SLA% for each team._x000D__x000D_
+_x000D__x000D_
+3. Alerts clear automatically the next time the cache refreshes (every 5 min) if the team's SLA% has recovered above the threshold. No manual dismissal needed — though users can manually dismiss from the UI to hide it for their session._x000D__x000D_
+_x000D__x000D_
 </t>
   </si>
   <si>
@@ -392,10 +403,10 @@
 Click the card to view individual application details.</t>
   </si>
   <si>
-    <t>Total applications received on the latest reporting date._x000D_
-_x000D_
-Counts distinct Application IDs where Date_ApplicationReceived falls on the reporting date._x000D_
-_x000D_
+    <t>Total applications received on the latest reporting date._x000D__x000D_
+_x000D__x000D_
+Counts distinct Application IDs where Date_ApplicationReceived falls on the reporting date._x000D__x000D_
+_x000D__x000D_
 Click the card to view individual application details.</t>
   </si>
   <si>
@@ -410,10 +421,10 @@
 Click the card to view individual application details.</t>
   </si>
   <si>
-    <t>Total applications approved by the funder on the latest reporting date._x000D_
-_x000D_
-Counts distinct Application IDs where Date_FunderApproval falls on the reporting date._x000D_
-_x000D_
+    <t>Total applications approved by the funder on the latest reporting date._x000D__x000D_
+_x000D__x000D_
+Counts distinct Application IDs where Date_FunderApproval falls on the reporting date._x000D__x000D_
+_x000D__x000D_
 Click the card to view individual application details.</t>
   </si>
   <si>
@@ -428,10 +439,10 @@
 Click the card to view individual application details.</t>
   </si>
   <si>
-    <t>Total loans settled on the latest reporting date._x000D_
-_x000D_
-Counts distinct Application IDs where Date_Settled falls on the reporting date._x000D_
-_x000D_
+    <t>Total loans settled on the latest reporting date._x000D__x000D_
+_x000D__x000D_
+Counts distinct Application IDs where Date_Settled falls on the reporting date._x000D__x000D_
+_x000D__x000D_
 Click the card to view individual application details.</t>
   </si>
   <si>
@@ -445,7 +456,7 @@
   </si>
   <si>
     <t>How often the dashboard silently fetches fresh data from the database.
-No page reload — all cards update in the background.
+No page reload - all cards update in the background.
 What refreshes:
 - KPI tiles
 - Team cards
@@ -454,25 +465,25 @@
 - Loan summary
 What does NOT auto-refresh:
 - History chart (only loads on login or Apply)
-Valid range: 1–60 minutes.
+Valid range: 1-60 minutes.
 Default: 5 minutes.</t>
   </si>
   <si>
-    <t>How often the dashboard silently fetches fresh data from the database._x000D_
-_x000D_
-No page reload — all cards update in the background._x000D_
-_x000D_
-What refreshes:_x000D_
-- KPI tiles_x000D_
-- Team cards_x000D_
-- Tasks list_x000D_
-- Alerts_x000D_
-- Loan summary_x000D_
-_x000D_
-What does NOT auto-refresh:_x000D_
-- History chart (only loads on login or Apply)_x000D_
-_x000D_
-Valid range: 1–60 minutes._x000D_
+    <t>How often the dashboard silently fetches fresh data from the database._x000D__x000D_
+_x000D__x000D_
+No page reload — all cards update in the background._x000D__x000D_
+_x000D__x000D_
+What refreshes:_x000D__x000D_
+- KPI tiles_x000D__x000D_
+- Team cards_x000D__x000D_
+- Tasks list_x000D__x000D_
+- Alerts_x000D__x000D_
+- Loan summary_x000D__x000D_
+_x000D__x000D_
+What does NOT auto-refresh:_x000D__x000D_
+- History chart (only loads on login or Apply)_x000D__x000D_
+_x000D__x000D_
+Valid range: 1–60 minutes._x000D__x000D_
 Default: 5 minutes.</t>
   </si>
   <si>
@@ -484,34 +495,34 @@
   <si>
     <t>How it works:
 A task turns amber before it breaches SLA.
-Task states (consumed = time spent ÷ SLA target):
-- Green — below threshold (on track)
-- Amber — at or above threshold (at risk)
-- Red — above 100% (overdue / breached)
+Task states (consumed = time spent / SLA target):
+- Green - below threshold (on track)
+- Amber - at or above threshold (at risk)
+- Red - above 100% (overdue / breached)
 Examples with a 4h SLA target:
-- 50% threshold → amber at 2h, red at 4h
-- 87.5% (default) → amber at 3.5h, red at 4h
+- 50% threshold -&gt; amber at 2h, red at 4h
+- 87.5% (default) -&gt; amber at 3.5h, red at 4h
 Applies to:
 - Task list row colours
 - Alerts panel drill-down
 - Warning alerts per team</t>
   </si>
   <si>
-    <t>How it works:_x000D_
-A task turns amber before it breaches SLA._x000D_
-_x000D_
-Task states (consumed = time spent ÷ SLA target):_x000D_
-- Green — below threshold (on track)_x000D_
-- Amber — at or above threshold (at risk)_x000D_
-- Red — above 100% (overdue / breached)_x000D_
-_x000D_
-Examples with a 4h SLA target:_x000D_
-- 50% threshold → amber at 2h, red at 4h_x000D_
-- 87.5% (default) → amber at 3.5h, red at 4h_x000D_
-_x000D_
-Applies to:_x000D_
-- Task list row colours_x000D_
-- Alerts panel drill-down_x000D_
+    <t>How it works:_x000D__x000D_
+A task turns amber before it breaches SLA._x000D__x000D_
+_x000D__x000D_
+Task states (consumed = time spent ÷ SLA target):_x000D__x000D_
+- Green — below threshold (on track)_x000D__x000D_
+- Amber — at or above threshold (at risk)_x000D__x000D_
+- Red — above 100% (overdue / breached)_x000D__x000D_
+_x000D__x000D_
+Examples with a 4h SLA target:_x000D__x000D_
+- 50% threshold → amber at 2h, red at 4h_x000D__x000D_
+- 87.5% (default) → amber at 3.5h, red at 4h_x000D__x000D_
+_x000D__x000D_
+Applies to:_x000D__x000D_
+- Task list row colours_x000D__x000D_
+- Alerts panel drill-down_x000D__x000D_
 - Warning alerts per team</t>
   </si>
   <si>
@@ -523,15 +534,15 @@
   <si>
     <t>Max number of tasks shown when you click into a team card or alert.
 Tasks are ranked by SLA consumption (highest first), so the most critical items appear at the top.
-Valid range: 1–100.
-Default: 10.</t>
-  </si>
-  <si>
-    <t>Max number of tasks shown when you click into a team card or alert._x000D_
-_x000D_
-Tasks are ranked by SLA consumption (highest first), so the most critical items appear at the top._x000D_
-_x000D_
-Valid range: 1–100._x000D_
+Valid range: 1-100.
+Default: 50.</t>
+  </si>
+  <si>
+    <t>Max number of tasks shown when you click into a team card or alert._x000D__x000D_
+_x000D__x000D_
+Tasks are ranked by SLA consumption (highest first), so the most critical items appear at the top._x000D__x000D_
+_x000D__x000D_
+Valid range: 1–100._x000D__x000D_
 Default: 50.</t>
   </si>
   <si>
@@ -546,6 +557,17 @@
 Date basis: Date Created.</t>
   </si>
   <si>
+    <t>Count of active tasks that have exceeded their SLA target.
+Rules:
+- Overdue when TotalHoursOnTask &gt; SLAInHours
+- Overdue when Current time &gt; SLAAdjustedDate
+- Overdue when TotalHoursOnTask &gt; SLA target hours in Setting tab
+Includes: Active
+Excluded: Cancelled; Completed tasks; Tasks where TotalHoursOnTask is null or = 0
+Date basis: Date Created.
+Target is configurable per team In Settings.</t>
+  </si>
+  <si>
     <t>Average TAT of ACTIVE tasks
 Rules:
 - avg TAT = avg TotalHoursOnTask 
@@ -565,10 +587,19 @@
     <t>Average TAT across completed tasks 
 Rules:
 - avg TAT = avg TotalHoursOnTask when not null
-- DateDiff (DateCreated, DateCompleted) in hours when TotalHoursOnTask is null and SLAAdjustedDate is set
+- DateDiff(DateCreated, DateCompleted) in hours when TotalHoursOnTask is null and SLAAdjustedDate is set
 Includes: Completed
 Excluded: Tasks where TotalHoursOnTask is null and SLAAdjustedDate is null
 Date basis: Date Created.</t>
+  </si>
+  <si>
+    <t>Count of completed tasks that exceeded their SLA target.
+Rules:
+- Overdue when TotalHoursOnTask &gt; SLAInHours
+- Overdue when DateCompleted &gt; SLAAdjustedDate
+Includes: Completed
+Excluded: Cancelled; Active tasks; Tasks where TotalHoursOnTask is null or = 0
+Date basis: Date Created</t>
   </si>
 </sst>
 </file>
@@ -586,7 +617,7 @@
     <font>
       <b/>
       <sz val="12"/>
-      <color theme="0"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -601,7 +632,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.499984740745262"/>
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -639,16 +670,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -656,15 +687,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1007,15 +1033,12 @@
   <dimension ref="A1:E25"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9" style="2"/>
-    <col min="2" max="2" width="22" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9" style="2"/>
-    <col min="4" max="4" width="82.625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="52.125" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="2"/>
+    <col min="1" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="83.625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="78.125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1028,422 +1051,423 @@
       <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="157.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="8" t="s">
+      <c r="E3" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="173.25" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+    <row r="4" spans="1:5" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="252" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+    </row>
+    <row r="5" spans="1:5" ht="220.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="7" t="s">
+    </row>
+    <row r="6" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="B6" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="E6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="7" t="s">
+    </row>
+    <row r="7" spans="1:5" ht="236.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="236.25" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="D7" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="E7" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="7" t="s">
+    </row>
+    <row r="8" spans="1:5" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="173.25" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="D8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E8" s="7" t="s">
+    </row>
+    <row r="9" spans="1:5" ht="220.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="252" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>20</v>
-      </c>
     </row>
     <row r="10" spans="1:5" ht="204.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
+      <c r="A10" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D10" s="7" t="s">
+      <c r="D10" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E10" s="7" t="s">
+      <c r="E10" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="204.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="7" t="s">
+      <c r="D11" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="E11" s="3" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="D12" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E12" s="7" t="s">
+      <c r="E12" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="236.25" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="7" t="s">
-        <v>29</v>
-      </c>
     </row>
     <row r="14" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="7" t="s">
+      <c r="D14" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E14" s="7" t="s">
+      <c r="E14" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="173.25" x14ac:dyDescent="0.25">
-      <c r="A15" s="6" t="s">
+    <row r="15" spans="1:5" ht="157.5" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="204.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+      <c r="D15" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="189" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="C16" s="6" t="s">
+      <c r="B16" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="7" t="s">
+      <c r="C16" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E16" s="7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" ht="252" x14ac:dyDescent="0.25">
-      <c r="A17" s="6" t="s">
+      <c r="D16" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="220.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C17" s="6" t="s">
+      <c r="B17" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D17" s="7" t="s">
+      <c r="C17" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" ht="189" x14ac:dyDescent="0.25">
-      <c r="A18" s="6" t="s">
+    </row>
+    <row r="18" spans="1:5" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="C18" s="6" t="s">
+      <c r="B18" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="C18" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E18" s="7" t="s">
+      <c r="D18" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="236.25" x14ac:dyDescent="0.25">
-      <c r="A19" s="6" t="s">
+    <row r="19" spans="1:5" ht="173.25" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="7" t="s">
+      <c r="D19" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="3" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    <row r="20" spans="1:5" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="D20" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="E20" s="7" t="s">
+      <c r="E20" s="3" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
-      <c r="A21" s="6" t="s">
+    <row r="21" spans="1:5" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="D21" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="E21" s="7" t="s">
+      <c r="E21" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="94.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="6" t="s">
+    <row r="22" spans="1:5" ht="78.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="D22" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="E22" s="7" t="s">
+      <c r="E22" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="267.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+    <row r="23" spans="1:5" ht="252" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="D23" s="7" t="s">
+      <c r="D23" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="E23" s="7" t="s">
+      <c r="E23" s="3" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="252" x14ac:dyDescent="0.25">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="D24" s="7" t="s">
+      <c r="D24" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="E24" s="7" t="s">
+      <c r="E24" s="3" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="126" x14ac:dyDescent="0.25">
-      <c r="A25" s="6" t="s">
+    <row r="25" spans="1:5" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="D25" s="7" t="s">
+      <c r="D25" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E25" s="7" t="s">
+      <c r="E25" s="3" t="s">
         <v>94</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:E3 A5:E7 A4:D4 A9:E14 A8:D8 A17:E25 A15:D15 A16:D16" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:E3 A6:E7 A4:C4 E4 A5:C5 E5 A10:E14 A8:C8 E8 A9:C9 E9 A19:E25 A15:C15 E15 A16:C16 E16 A17:C17 E17 A18:C18 E18" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1471,7 +1495,7 @@
     </row>
     <row r="3" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3">
         <v>4</v>

</xml_diff>